<commit_message>
--ignore filters based ONLY on values in new.xlsx
</commit_message>
<xml_diff>
--- a/test_data/xlsx_diff/old.xlsx
+++ b/test_data/xlsx_diff/old.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/ICTV/ICTVvmrUpdate/test_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/curtish/Documents/ICTV/ICTVvmr-update/test_data/xlsx_diff/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{15B06D73-F172-EB46-A274-23F39E493DD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F80F663-7483-9340-91CE-D62AA1C83F7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3340" yWindow="3660" windowWidth="25640" windowHeight="14440" xr2:uid="{295F2116-0CB0-C048-85BD-FF48A684A5E6}"/>
   </bookViews>
@@ -36,12 +36,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>fred</t>
   </si>
   <si>
     <t>jane</t>
+  </si>
+  <si>
+    <t>ignore this line</t>
+  </si>
+  <si>
+    <t>ignore doesn’t' work on values in "old.xlsx" - filters only on new values!</t>
   </si>
 </sst>
 </file>
@@ -413,17 +419,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2041A03-887F-474F-AA34-B33A16095E0E}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>